<commit_message>
Update - Concept files
</commit_message>
<xml_diff>
--- a/ideas_ressources_files/plant_port_checklist.xlsx
+++ b/ideas_ressources_files/plant_port_checklist.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\pvz_lawnmageddon\ideas_ressources_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\rogue_garden\ideas_ressources_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9343E672-D449-4CDD-A8BE-02777188EA1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4236A5C9-F3BF-463E-82F4-E1213358E3B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11448" yWindow="0" windowWidth="11688" windowHeight="12336" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PvZ 1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1811" uniqueCount="953">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1813" uniqueCount="955">
   <si>
     <t>Origin Name</t>
   </si>
@@ -2454,9 +2454,6 @@
     <t>Primal Umbrella Leaf</t>
   </si>
   <si>
-    <t>Watered Vase</t>
-  </si>
-  <si>
     <t>Feral Sunflower</t>
   </si>
   <si>
@@ -2893,6 +2890,15 @@
   </si>
   <si>
     <t>Button-shroom</t>
+  </si>
+  <si>
+    <t>Three Pod</t>
+  </si>
+  <si>
+    <t>Water Vase</t>
+  </si>
+  <si>
+    <t>Shadow Repeater</t>
   </si>
 </sst>
 </file>
@@ -3319,7 +3325,7 @@
         <v>3</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -3441,7 +3447,7 @@
         <v>1</v>
       </c>
       <c r="G8" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -4223,7 +4229,7 @@
         <v>1</v>
       </c>
       <c r="G54" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -4566,7 +4572,7 @@
         <v>1</v>
       </c>
       <c r="G74" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -4622,7 +4628,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
@@ -4633,13 +4639,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="C2" s="7" t="b">
         <v>1</v>
       </c>
       <c r="E2" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -4647,7 +4653,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="C3" s="7" t="b">
         <v>0</v>
@@ -4661,7 +4667,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="C4" s="7" t="b">
         <v>0</v>
@@ -4675,7 +4681,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="C5" s="7" t="b">
         <v>1</v>
@@ -4689,7 +4695,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>806</v>
+        <v>953</v>
       </c>
       <c r="C6" s="7" t="b">
         <v>0</v>
@@ -4748,7 +4754,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="E10" s="7" t="b">
         <v>0</v>
@@ -4762,7 +4768,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="E11" s="7" t="b">
         <v>0</v>
@@ -4776,7 +4782,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="E12" s="7" t="b">
         <v>0</v>
@@ -4790,7 +4796,7 @@
         <v>1</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="E13" s="7" t="b">
         <v>0</v>
@@ -4807,7 +4813,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -4821,7 +4827,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -4835,10 +4841,10 @@
         <v>1</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>946</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="b">
         <v>0</v>
       </c>
@@ -4846,10 +4852,13 @@
         <v>0</v>
       </c>
       <c r="E17" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="b">
         <v>0</v>
       </c>
@@ -4857,10 +4866,13 @@
         <v>0</v>
       </c>
       <c r="E18" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="b">
         <v>0</v>
       </c>
@@ -4871,7 +4883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="b">
         <v>0</v>
       </c>
@@ -4882,7 +4894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="b">
         <v>0</v>
       </c>
@@ -4893,7 +4905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="b">
         <v>0</v>
       </c>
@@ -4904,7 +4916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="b">
         <v>0</v>
       </c>
@@ -4915,7 +4927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="b">
         <v>0</v>
       </c>
@@ -4926,7 +4938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="b">
         <v>0</v>
       </c>
@@ -4937,7 +4949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="b">
         <v>0</v>
       </c>
@@ -4948,7 +4960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="b">
         <v>0</v>
       </c>
@@ -4959,7 +4971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="b">
         <v>0</v>
       </c>
@@ -4970,7 +4982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="7" t="b">
         <v>0</v>
       </c>
@@ -4981,7 +4993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="b">
         <v>0</v>
       </c>
@@ -4992,7 +5004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="b">
         <v>0</v>
       </c>
@@ -5003,7 +5015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="b">
         <v>0</v>
       </c>
@@ -5498,7 +5510,7 @@
         <v>3</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -5705,7 +5717,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -5786,7 +5798,7 @@
         <v>3</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -6108,7 +6120,7 @@
         <v>3</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -6626,7 +6638,7 @@
     </row>
     <row r="32" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>166</v>
@@ -6672,7 +6684,7 @@
         <v>1</v>
       </c>
       <c r="G34" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -6791,7 +6803,7 @@
         <v>1</v>
       </c>
       <c r="G41" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -6825,7 +6837,7 @@
         <v>1</v>
       </c>
       <c r="G43" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -6842,7 +6854,7 @@
         <v>1</v>
       </c>
       <c r="G44" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -7003,7 +7015,7 @@
     </row>
     <row r="54" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>60</v>
@@ -7321,7 +7333,7 @@
         <v>1</v>
       </c>
       <c r="G72" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -7494,7 +7506,7 @@
         <v>1</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="G82" s="7" t="b">
         <v>0</v>
@@ -8004,7 +8016,7 @@
         <v>221</v>
       </c>
       <c r="C112" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E112" s="7" t="b">
         <v>1</v>
@@ -8435,7 +8447,7 @@
         <v>1</v>
       </c>
       <c r="G137" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="138" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -8452,7 +8464,7 @@
         <v>1</v>
       </c>
       <c r="G138" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="139" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -8622,7 +8634,7 @@
         <v>1</v>
       </c>
       <c r="G148" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -8656,7 +8668,7 @@
         <v>1</v>
       </c>
       <c r="G150" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="151" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -8916,7 +8928,7 @@
     </row>
     <row r="166" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="5" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="B166" s="6" t="s">
         <v>221</v>
@@ -8933,7 +8945,7 @@
     </row>
     <row r="167" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A167" s="5" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="B167" s="6" t="s">
         <v>221</v>
@@ -8945,7 +8957,7 @@
         <v>1</v>
       </c>
       <c r="F167" s="5" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="G167" s="7" t="b">
         <v>0</v>
@@ -8959,7 +8971,7 @@
         <v>134</v>
       </c>
       <c r="C168" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E168" s="7" t="b">
         <v>1</v>
@@ -9046,7 +9058,7 @@
         <v>3</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -9202,7 +9214,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="G10" s="7" t="b">
         <v>1</v>
@@ -9511,7 +9523,7 @@
         <v>1</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="G28" s="7" t="b">
         <v>0</v>
@@ -9990,7 +10002,7 @@
         <v>1</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="G56" s="7" t="b">
         <v>0</v>
@@ -10151,7 +10163,7 @@
     </row>
     <row r="66" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>361</v>
@@ -10270,7 +10282,7 @@
     </row>
     <row r="73" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B73" s="6" t="s">
         <v>361</v>
@@ -10338,7 +10350,7 @@
     </row>
     <row r="77" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="B77" s="6" t="s">
         <v>361</v>
@@ -10350,7 +10362,7 @@
         <v>1</v>
       </c>
       <c r="F77" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="G77" s="7" t="b">
         <v>0</v>
@@ -10594,7 +10606,7 @@
         <v>1</v>
       </c>
       <c r="F91" s="5" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="G91" s="7" t="b">
         <v>0</v>
@@ -10750,7 +10762,7 @@
         <v>1</v>
       </c>
       <c r="F100" s="5" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="G100" s="7" t="b">
         <v>0</v>
@@ -10911,7 +10923,7 @@
     </row>
     <row r="110" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="B110" s="6" t="s">
         <v>437</v>
@@ -11016,7 +11028,7 @@
     </row>
     <row r="116" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="5" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="B116" s="6" t="s">
         <v>437</v>
@@ -11099,7 +11111,7 @@
         <v>1</v>
       </c>
       <c r="F120" s="5" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G120" s="7" t="b">
         <v>0</v>
@@ -11136,7 +11148,7 @@
         <v>1</v>
       </c>
       <c r="F122" s="5" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="G122" s="7" t="b">
         <v>0</v>
@@ -11156,7 +11168,7 @@
         <v>1</v>
       </c>
       <c r="F123" s="5" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G123" s="7" t="b">
         <v>0</v>
@@ -11244,7 +11256,7 @@
         <v>1</v>
       </c>
       <c r="F128" s="5" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="G128" s="7" t="b">
         <v>0</v>
@@ -11473,7 +11485,7 @@
     </row>
     <row r="142" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="5" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="B142" s="6" t="s">
         <v>353</v>
@@ -11566,7 +11578,7 @@
         <v>3</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -11594,7 +11606,7 @@
         <v>769</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="C3" s="7" t="b">
         <v>1</v>
@@ -11608,10 +11620,10 @@
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C4" s="7" t="b">
         <v>0</v>
@@ -11625,10 +11637,10 @@
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C5" s="7" t="b">
         <v>0</v>
@@ -11642,10 +11654,10 @@
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C6" s="7" t="b">
         <v>0</v>
@@ -11659,10 +11671,10 @@
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
+        <v>819</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>820</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>821</v>
       </c>
       <c r="C7" s="7" t="b">
         <v>0</v>
@@ -11676,10 +11688,10 @@
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C8" s="7" t="b">
         <v>0</v>
@@ -11710,10 +11722,10 @@
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C10" s="7" t="b">
         <v>0</v>
@@ -11727,10 +11739,10 @@
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C11" s="7" t="b">
         <v>0</v>
@@ -11744,10 +11756,10 @@
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C12" s="7" t="b">
         <v>0</v>
@@ -11778,10 +11790,10 @@
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C14" s="7" t="b">
         <v>0</v>
@@ -11795,10 +11807,10 @@
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C15" s="7" t="b">
         <v>0</v>
@@ -11812,10 +11824,10 @@
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C16" s="7" t="b">
         <v>0</v>
@@ -11829,10 +11841,10 @@
     </row>
     <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C17" s="7" t="b">
         <v>0</v>
@@ -11846,10 +11858,10 @@
     </row>
     <row r="18" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
+        <v>822</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>823</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>824</v>
       </c>
       <c r="C18" s="7" t="b">
         <v>0</v>
@@ -11880,10 +11892,10 @@
     </row>
     <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C20" s="7" t="b">
         <v>0</v>
@@ -11931,10 +11943,10 @@
     </row>
     <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C23" s="7" t="b">
         <v>0</v>
@@ -11948,10 +11960,10 @@
     </row>
     <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C24" s="7" t="b">
         <v>0</v>
@@ -11965,10 +11977,10 @@
     </row>
     <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C25" s="7" t="b">
         <v>0</v>
@@ -12084,10 +12096,10 @@
     </row>
     <row r="32" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C32" s="7" t="b">
         <v>0</v>
@@ -12135,10 +12147,10 @@
     </row>
     <row r="35" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="C35" s="7" t="b">
         <v>0</v>
@@ -12169,10 +12181,10 @@
     </row>
     <row r="37" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C37" s="7" t="b">
         <v>0</v>
@@ -12186,10 +12198,10 @@
     </row>
     <row r="38" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C38" s="7" t="b">
         <v>0</v>
@@ -12203,10 +12215,10 @@
     </row>
     <row r="39" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C39" s="7" t="b">
         <v>0</v>
@@ -12220,10 +12232,10 @@
     </row>
     <row r="40" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C40" s="7" t="b">
         <v>0</v>
@@ -12237,10 +12249,10 @@
     </row>
     <row r="41" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C41" s="7" t="b">
         <v>0</v>
@@ -12254,10 +12266,10 @@
     </row>
     <row r="42" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C42" s="7" t="b">
         <v>0</v>
@@ -12288,10 +12300,10 @@
     </row>
     <row r="44" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C44" s="7" t="b">
         <v>0</v>
@@ -12305,10 +12317,10 @@
     </row>
     <row r="45" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C45" s="7" t="b">
         <v>0</v>
@@ -12407,10 +12419,10 @@
     </row>
     <row r="51" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C51" s="7" t="b">
         <v>0</v>
@@ -12424,10 +12436,10 @@
     </row>
     <row r="52" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C52" s="7" t="b">
         <v>0</v>
@@ -12441,10 +12453,10 @@
     </row>
     <row r="53" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C53" s="7" t="b">
         <v>0</v>
@@ -12458,10 +12470,10 @@
     </row>
     <row r="54" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C54" s="7" t="b">
         <v>0</v>
@@ -12475,10 +12487,10 @@
     </row>
     <row r="55" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C55" s="7" t="b">
         <v>0</v>
@@ -12487,7 +12499,7 @@
         <v>1</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G55" s="7" t="b">
         <v>0</v>
@@ -12512,10 +12524,10 @@
     </row>
     <row r="57" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C57" s="7" t="b">
         <v>0</v>
@@ -12529,10 +12541,10 @@
     </row>
     <row r="58" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C58" s="7" t="b">
         <v>0</v>
@@ -12546,10 +12558,10 @@
     </row>
     <row r="59" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C59" s="7" t="b">
         <v>0</v>
@@ -12563,10 +12575,10 @@
     </row>
     <row r="60" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C60" s="7" t="b">
         <v>0</v>
@@ -12580,10 +12592,10 @@
     </row>
     <row r="61" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C61" s="7" t="b">
         <v>0</v>
@@ -12597,10 +12609,10 @@
     </row>
     <row r="62" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C62" s="7" t="b">
         <v>0</v>
@@ -12614,10 +12626,10 @@
     </row>
     <row r="63" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C63" s="7" t="b">
         <v>0</v>
@@ -12631,10 +12643,10 @@
     </row>
     <row r="64" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C64" s="7" t="b">
         <v>0</v>
@@ -12648,10 +12660,10 @@
     </row>
     <row r="65" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="C65" s="7" t="b">
         <v>0</v>
@@ -12665,10 +12677,10 @@
     </row>
     <row r="66" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="C66" s="7" t="b">
         <v>0</v>
@@ -12682,10 +12694,10 @@
     </row>
     <row r="67" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="C67" s="7" t="b">
         <v>0</v>
@@ -12702,7 +12714,7 @@
         <v>556</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C68" s="7" t="b">
         <v>0</v>
@@ -12716,10 +12728,10 @@
     </row>
     <row r="69" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C69" s="7" t="b">
         <v>0</v>
@@ -12733,10 +12745,10 @@
     </row>
     <row r="70" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C70" s="7" t="b">
         <v>0</v>
@@ -12750,10 +12762,10 @@
     </row>
     <row r="71" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C71" s="7" t="b">
         <v>0</v>
@@ -12767,10 +12779,10 @@
     </row>
     <row r="72" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C72" s="7" t="b">
         <v>0</v>
@@ -12784,10 +12796,10 @@
     </row>
     <row r="73" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C73" s="7" t="b">
         <v>0</v>
@@ -12801,10 +12813,10 @@
     </row>
     <row r="74" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C74" s="7" t="b">
         <v>0</v>
@@ -12818,10 +12830,10 @@
     </row>
     <row r="75" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C75" s="7" t="b">
         <v>0</v>
@@ -12835,10 +12847,10 @@
     </row>
     <row r="76" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C76" s="7" t="b">
         <v>0</v>
@@ -12847,7 +12859,7 @@
         <v>1</v>
       </c>
       <c r="F76" s="5" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="G76" s="7" t="b">
         <v>0</v>
@@ -12855,10 +12867,10 @@
     </row>
     <row r="77" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C77" s="7" t="b">
         <v>0</v>
@@ -12872,10 +12884,10 @@
     </row>
     <row r="78" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C78" s="7" t="b">
         <v>0</v>
@@ -12889,10 +12901,10 @@
     </row>
     <row r="79" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="C79" s="7" t="b">
         <v>0</v>
@@ -12906,10 +12918,10 @@
     </row>
     <row r="80" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="C80" s="7" t="b">
         <v>0</v>
@@ -12923,10 +12935,10 @@
     </row>
     <row r="81" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C81" s="7" t="b">
         <v>0</v>
@@ -12940,10 +12952,10 @@
     </row>
     <row r="82" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
+        <v>920</v>
+      </c>
+      <c r="B82" s="6" t="s">
         <v>921</v>
-      </c>
-      <c r="B82" s="6" t="s">
-        <v>922</v>
       </c>
       <c r="C82" s="7" t="b">
         <v>0</v>
@@ -12957,10 +12969,10 @@
     </row>
     <row r="83" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="5" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="C83" s="7" t="b">
         <v>0</v>
@@ -12974,10 +12986,10 @@
     </row>
     <row r="84" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="C84" s="7" t="b">
         <v>0</v>
@@ -12991,10 +13003,10 @@
     </row>
     <row r="85" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="5" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="C85" s="7" t="b">
         <v>0</v>
@@ -13008,10 +13020,10 @@
     </row>
     <row r="86" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="5" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C86" s="7" t="b">
         <v>0</v>
@@ -13025,10 +13037,10 @@
     </row>
     <row r="87" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="5" t="s">
+        <v>889</v>
+      </c>
+      <c r="B87" s="6" t="s">
         <v>890</v>
-      </c>
-      <c r="B87" s="6" t="s">
-        <v>891</v>
       </c>
       <c r="C87" s="7" t="b">
         <v>0</v>
@@ -13042,10 +13054,10 @@
     </row>
     <row r="88" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="5" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C88" s="7" t="b">
         <v>0</v>
@@ -13059,10 +13071,10 @@
     </row>
     <row r="89" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="5" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="C89" s="7" t="b">
         <v>0</v>
@@ -13076,10 +13088,10 @@
     </row>
     <row r="90" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="5" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="C90" s="7" t="b">
         <v>0</v>
@@ -13093,10 +13105,10 @@
     </row>
     <row r="91" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="C91" s="7" t="b">
         <v>0</v>
@@ -13110,10 +13122,10 @@
     </row>
     <row r="92" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="5" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="C92" s="7" t="b">
         <v>0</v>
@@ -13127,10 +13139,10 @@
     </row>
     <row r="93" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="C93" s="7" t="b">
         <v>0</v>
@@ -13144,10 +13156,10 @@
     </row>
     <row r="94" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="5" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="C94" s="7" t="b">
         <v>0</v>
@@ -13161,10 +13173,10 @@
     </row>
     <row r="95" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C95" s="7" t="b">
         <v>0</v>
@@ -13178,10 +13190,10 @@
     </row>
     <row r="96" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="5" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="C96" s="7" t="b">
         <v>0</v>
@@ -13195,10 +13207,10 @@
     </row>
     <row r="97" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="5" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C97" s="7" t="b">
         <v>0</v>
@@ -13207,7 +13219,7 @@
         <v>1</v>
       </c>
       <c r="F97" s="5" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="G97" s="7" t="b">
         <v>0</v>
@@ -13215,10 +13227,10 @@
     </row>
     <row r="98" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="C98" s="7" t="b">
         <v>0</v>
@@ -13227,7 +13239,7 @@
         <v>1</v>
       </c>
       <c r="F98" s="5" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="G98" s="7" t="b">
         <v>0</v>
@@ -13235,10 +13247,10 @@
     </row>
     <row r="99" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="C99" s="7" t="b">
         <v>0</v>
@@ -13252,10 +13264,10 @@
     </row>
     <row r="100" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="5" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="C100" s="7" t="b">
         <v>0</v>
@@ -13269,10 +13281,10 @@
     </row>
     <row r="101" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="B101" s="6" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="C101" s="7" t="b">
         <v>0</v>
@@ -13286,10 +13298,10 @@
     </row>
     <row r="102" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="C102" s="7" t="b">
         <v>0</v>
@@ -13303,10 +13315,10 @@
     </row>
     <row r="103" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="5" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="C103" s="7" t="b">
         <v>0</v>
@@ -13320,10 +13332,10 @@
     </row>
     <row r="104" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="5" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="C104" s="7" t="b">
         <v>0</v>
@@ -13337,10 +13349,10 @@
     </row>
     <row r="105" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="5" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="B105" s="6" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C105" s="7" t="b">
         <v>0</v>
@@ -13354,10 +13366,10 @@
     </row>
     <row r="106" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="5" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="C106" s="7" t="b">
         <v>0</v>
@@ -13371,10 +13383,10 @@
     </row>
     <row r="107" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="5" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="C107" s="7" t="b">
         <v>0</v>
@@ -13388,10 +13400,10 @@
     </row>
     <row r="108" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="5" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="B108" s="6" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C108" s="7" t="b">
         <v>0</v>
@@ -13405,10 +13417,10 @@
     </row>
     <row r="109" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="5" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="B109" s="6" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="C109" s="7" t="b">
         <v>0</v>
@@ -13422,10 +13434,10 @@
     </row>
     <row r="110" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="B110" s="6" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="C110" s="7" t="b">
         <v>0</v>
@@ -13439,10 +13451,10 @@
     </row>
     <row r="111" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="5" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C111" s="7" t="b">
         <v>0</v>
@@ -13459,7 +13471,7 @@
         <v>316</v>
       </c>
       <c r="B112" s="6" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C112" s="7" t="b">
         <v>0</v>
@@ -13473,10 +13485,10 @@
     </row>
     <row r="113" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="5" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C113" s="7" t="b">
         <v>0</v>
@@ -13490,10 +13502,10 @@
     </row>
     <row r="114" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="5" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="B114" s="6" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C114" s="7" t="b">
         <v>0</v>
@@ -13507,10 +13519,10 @@
     </row>
     <row r="115" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="5" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="B115" s="6" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="C115" s="7" t="b">
         <v>0</v>
@@ -13524,10 +13536,10 @@
     </row>
     <row r="116" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="5" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="B116" s="6" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C116" s="7" t="b">
         <v>0</v>
@@ -13541,10 +13553,10 @@
     </row>
     <row r="117" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="5" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="B117" s="6" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="C117" s="7" t="b">
         <v>0</v>
@@ -13601,7 +13613,7 @@
         <v>3</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -14035,7 +14047,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -14466,7 +14478,7 @@
     </row>
     <row r="52" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="B52" s="6" t="s">
         <v>582</v>
@@ -14525,7 +14537,7 @@
         <v>3</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -15415,7 +15427,7 @@
         <v>1</v>
       </c>
       <c r="G53" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -15650,7 +15662,7 @@
         <v>1</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="E67" s="7" t="b">
         <v>0</v>
@@ -16247,7 +16259,7 @@
         <v>3</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -16669,7 +16681,7 @@
         <v>605</v>
       </c>
       <c r="C26" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E26" s="7" t="b">
         <v>1</v>
@@ -17003,7 +17015,7 @@
     </row>
     <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>638</v>
@@ -17018,7 +17030,7 @@
         <v>1</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -17046,7 +17058,7 @@
         <v>638</v>
       </c>
       <c r="C48" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E48" s="7" t="b">
         <v>1</v>
@@ -17256,7 +17268,7 @@
         <v>1</v>
       </c>
       <c r="F60" s="5" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="G60" s="7" t="b">
         <v>0</v>
@@ -17735,7 +17747,7 @@
         <v>1</v>
       </c>
       <c r="G88" s="7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -17953,7 +17965,7 @@
         <v>0</v>
       </c>
       <c r="E101" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G101" s="7" t="b">
         <v>0</v>
@@ -18160,7 +18172,7 @@
         <v>1</v>
       </c>
       <c r="F113" s="5" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="G113" s="7" t="b">
         <v>0</v>
@@ -18263,7 +18275,7 @@
         <v>0</v>
       </c>
       <c r="E119" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G119" s="7" t="b">
         <v>0</v>
@@ -19019,7 +19031,7 @@
     </row>
     <row r="164" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A164" s="5" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="B164" s="6" t="s">
         <v>638</v>

</xml_diff>

<commit_message>
Added - First batch of New Artstyle plants
</commit_message>
<xml_diff>
--- a/ideas_ressources_files/plant_port_checklist.xlsx
+++ b/ideas_ressources_files/plant_port_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Documents\- Games\PvZ Game Concept\rogue_garden\ideas_ressources_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4236A5C9-F3BF-463E-82F4-E1213358E3B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D11E2328-07F8-4A99-BF26-2DC94715B3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PvZ 1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1813" uniqueCount="955">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1815" uniqueCount="956">
   <si>
     <t>Origin Name</t>
   </si>
@@ -2899,6 +2899,9 @@
   </si>
   <si>
     <t>Shadow Repeater</t>
+  </si>
+  <si>
+    <t>Fire Pea</t>
   </si>
 </sst>
 </file>
@@ -6381,7 +6384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>136</v>
       </c>
@@ -6398,7 +6401,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>139</v>
       </c>
@@ -6415,7 +6418,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>138</v>
       </c>
@@ -6432,7 +6435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>204</v>
       </c>
@@ -6449,7 +6452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>200</v>
       </c>
@@ -6462,11 +6465,17 @@
       <c r="E21" s="7" t="b">
         <v>1</v>
       </c>
+      <c r="F21" s="5" t="s">
+        <v>955</v>
+      </c>
       <c r="G21" s="7" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H21" s="5" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>196</v>
       </c>
@@ -6483,7 +6492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>195</v>
       </c>
@@ -6500,7 +6509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>199</v>
       </c>
@@ -6517,7 +6526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>203</v>
       </c>
@@ -6534,7 +6543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>201</v>
       </c>
@@ -6551,7 +6560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>194</v>
       </c>
@@ -6568,7 +6577,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>198</v>
       </c>
@@ -6585,7 +6594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>202</v>
       </c>
@@ -6602,7 +6611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>197</v>
       </c>
@@ -6619,7 +6628,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>162</v>
       </c>
@@ -6636,7 +6645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>807</v>
       </c>

</xml_diff>